<commit_message>
docs(synthea): showcase window-function derivation in the report table
Add a `latest_a1c` column to member_quality_summary whose derivation uses a
window-function candidate (row_filter + order_by + select_columns) and a
survivorship default_condition — demonstrating the derivation fields now
preserved end-to-end through the Excel round-trip. Regenerate specs, UMFs, and
the rendered guidebook.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/synthea/specs/claims.xlsx
+++ b/examples/synthea/specs/claims.xlsx
@@ -2121,7 +2121,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J1"/>
+  <dimension ref="A1:Q1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2162,15 +2162,50 @@
       </c>
       <c r="H1" s="5" t="inlineStr">
         <is>
+          <t>Row Filter</t>
+        </is>
+      </c>
+      <c r="I1" s="5" t="inlineStr">
+        <is>
+          <t>Order By</t>
+        </is>
+      </c>
+      <c r="J1" s="5" t="inlineStr">
+        <is>
+          <t>Select Columns</t>
+        </is>
+      </c>
+      <c r="K1" s="5" t="inlineStr">
+        <is>
+          <t>Join Via</t>
+        </is>
+      </c>
+      <c r="L1" s="5" t="inlineStr">
+        <is>
           <t>Reason</t>
         </is>
       </c>
-      <c r="I1" s="5" t="inlineStr">
-        <is>
-          <t>Strategy</t>
-        </is>
-      </c>
-      <c r="J1" s="5" t="inlineStr">
+      <c r="M1" s="5" t="inlineStr">
+        <is>
+          <t>Derivation Strategy</t>
+        </is>
+      </c>
+      <c r="N1" s="5" t="inlineStr">
+        <is>
+          <t>Survivorship Strategy</t>
+        </is>
+      </c>
+      <c r="O1" s="5" t="inlineStr">
+        <is>
+          <t>Default Value</t>
+        </is>
+      </c>
+      <c r="P1" s="5" t="inlineStr">
+        <is>
+          <t>Default Condition</t>
+        </is>
+      </c>
+      <c r="Q1" s="5" t="inlineStr">
         <is>
           <t>Survivorship Explanation</t>
         </is>

</xml_diff>